<commit_message>
dcos: actuaizlacion de la documentacion
</commit_message>
<xml_diff>
--- a/data/outputs/diagnostico_matcheo.xlsx
+++ b/data/outputs/diagnostico_matcheo.xlsx
@@ -442,7 +442,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-03-26 11:55:55</t>
+          <t>2026-03-27 16:49:56</t>
         </is>
       </c>
     </row>
@@ -2689,7 +2689,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Permisos de Embarque MOA Reingenieria</t>
+          <t>Permisos de Embarque MOA Reingeniería</t>
         </is>
       </c>
       <c r="C16" t="b">

</xml_diff>